<commit_message>
Save narrative system and UI progress
</commit_message>
<xml_diff>
--- a/Assets/ConfigTables/Data/Text.xlsx
+++ b/Assets/ConfigTables/Data/Text.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Text" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Text" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,11 +27,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00666666"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -43,11 +39,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004F81BD"/>
+        <fgColor rgb="00D9E2F3"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -55,20 +51,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -435,13 +443,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -467,104 +475,1538 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>##type</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>##group</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>##</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>策划约定的直观文本 key</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>实际显示文本</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>策划备注</t>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>comment</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="n"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>npc.a.name</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>艾德里安</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>A · 短工佣人，出身寒微</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>npc.a.desc</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>在王都打短工的年轻人，读过几本禁书。</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>A 角色描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>npc.b.name</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>塞西莉亚</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>B · 没落王选者家的小姐</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>npc.b.desc</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>家道中落的贵族小姐，不甘于被安排的婚事。</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>B 角色描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>npc.c.name</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>朱利安</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>C · 普通王选者家族的少爷</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>npc.c.desc</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>出身体面的年轻贵族，一心想娶塞西莉亚。</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>C 角色描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>npc.d.name</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>老伯爵瓦尔蒙</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>D · 塞西莉亚的父亲</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>npc.d.desc</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>固执的旧贵族，把家族的体面看得比女儿重要。</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>D 角色描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>player.name</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>你</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>玩家 · 咖啡馆的旁观者</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>player.desc</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>你坐在咖啡馆的角落，看着这一切发生。你可以插手，也可以只是看着。</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>玩家描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>world.name</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>奥尔狄亚王国</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>世界观</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>world.desc</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>一个王权将倾的王国。咖啡馆里，新旧思想正在交锋。</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>世界描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>bar.a.thought.name</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>进步思想</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>A 的思想觉悟</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>bar.a.trust_b.name</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>A对B的爱慕</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>A 对 B 的感情</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>bar.a.respect_c.name</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>A对C的敬服</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>A 对 C 的态度</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>bar.b.trust_a.name</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>B对A的爱慕</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>B 对 A 的感情</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>bar.b.trust_c.name</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>B对C的情谊</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>B 对 C 的感情</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>bar.b.trust_d.name</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>B对父亲的信任</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>B 对 D 的信任</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>bar.b.rebel.name</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>B的叛逆</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>B 的叛逆程度</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>bar.c.wealth.name</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>C的家产</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>C 的家产与地位</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>bar.c.trust_b.name</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>C对B的爱慕</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>C 对 B 的感情</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>bar.stability.name</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>王国稳定</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>王国的稳定程度</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>bar.calendar.name</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>第几天</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n"/>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>ev.act.meet.title</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>咖啡馆的私语</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n"/>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>ev.act.meet.p1</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>你替艾德里安和塞西莉亚在咖啡馆后座留了位置。</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>ev.act.meet.p2</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>两人说了很久的话。离开时，塞西莉亚的脸上有一点笑意。</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>ev.act.cwithb.title</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>让让他们独处</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>ev.act.cwithb.p1</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>你替朱利安制造了一个和塞西莉亚独处的下午。</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>ev.act.cwithb.p2</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>他讲了些得体的笑话，塞西莉亚礼貌地听着。</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n"/>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>ev.act.salon.title</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>改革派沙龙</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n"/>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>ev.act.salon.p1</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>你把艾德里安带进了改革派的沙龙。</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n"/>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>ev.act.salon.p2</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>他听得很认真，末了问了一句让全场安静下来的话。</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n"/>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>ev.act.peer.title</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>伯爵的关系</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n"/>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>ev.act.peer.p1</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>你替朱利安搭上了伯爵的门路。</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n"/>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>ev.act.peer.p2</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>一个月后，他谋到了一个体面的职位。</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>ev.talk.cafe.title</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>咖啡馆的午后</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n"/>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>ev.talk.cafe.p1</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>塞西莉亚坐在窗边，用勺子搅着已经凉掉的咖啡。她说：「你说，人是不是只能过一种人生。」</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n"/>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>choice.talk.cafe.a</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>「你可以选别人没走过的那条。」</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n"/>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>choice.talk.cafe.b</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>「回去吧，别让你父亲担心。」</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n"/>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>choice.talk.cafe.c</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>「时代要变了，你我都看得见。」</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n"/>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>ev.ab.swear.title</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>私定终生</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n"/>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>ev.ab.swear.p1</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>塞西莉亚摘下颈上那枚旧坠子，塞进艾德里安手里。</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n"/>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>ev.ab.swear.p2</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>「等春天，我们就走。」</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n"/>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>ev.ab.swear.p3</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>咖啡馆的灯影在窗上晃了一下，谁也没有再说话。</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n"/>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>ev.bc.swear.title</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>门当户对</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n"/>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>ev.bc.swear.p1</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>朱利安跪在塞西莉亚面前，捧出家族的戒指。</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n"/>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>ev.bc.swear.p2</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>「我会给你一个体面的家。」</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n"/>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>ev.bc.swear.p3</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>塞西莉亚看了很久，最后点了点头。</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n"/>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>ev.standoff.title</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>三人的对峙</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n"/>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>ev.standoff.p1</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>咖啡馆打烊了，只剩下三个人和一盏灯。</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n"/>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>ev.standoff.p2</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>「你凭什么？」朱利安说。艾德里安没有回答。</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n"/>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>ev.standoff.p3</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>塞西莉亚站在中间，谁也没有看。</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n"/>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>ev.comrade.title</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>同志</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n"/>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>ev.comrade.p1</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>艾德里安把一本小册子推到朱利安面前。</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n"/>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>ev.comrade.p2</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>朱利安读了一夜。天亮时他说：「你说得对。」</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n"/>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>ev.prison.title</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>冤狱</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n"/>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>ev.prison.p1</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>塞西莉亚被指控窝藏禁书，押进了圣西尔万的黑牢。</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n"/>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>ev.prison.p2</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>老伯爵在门外站了很久，最终没有进去。</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n"/>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>ev.rescue.title</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>捞人</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n"/>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>ev.rescue.p1</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>你动用了积攒多年的关系。</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n"/>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>ev.rescue.p2</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>三天后，塞西莉亚从牢里走了出来，瘦了一圈。</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n"/>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>ev.dq1.title</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>第一次顶撞</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n"/>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>ev.dq1.p1</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>「我不嫁。」塞西莉亚说。</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n"/>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>ev.dq1.p2</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>老伯爵把茶杯顿在桌上，没有再说一个字。</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n"/>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>ev.dq2.title</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>第二次顶撞</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n"/>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>ev.dq2.p1</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>「你从来只想着你那个姓氏！」</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n"/>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>ev.dq2.p2</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>这一次，塞西莉亚摔门而出。</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n"/>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>ev.dqn.title</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>沉默的餐桌</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n"/>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>ev.dqn.p1</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>父女二人隔着一张长桌吃饭，全程没有人开口。</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n"/>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>ev.elope.title</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>私奔</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n"/>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>ev.elope.p1</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>没有婚礼，没有嫁妆。两个人趁着夜色出了城门。</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n"/>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>ev.elope.p2</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>塞西莉亚回头看了一眼，老伯爵的宅邸没有一盏灯是亮的。</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n"/>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>ev.flee.title</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>家族的出走</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n"/>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>ev.flee.p1</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>恐怖统治的前夜，瓦尔蒙一家收拾了细软，连夜离开了奥尔狄亚。</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n"/>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>ev.flee.p2</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>塞西莉亚什么也没带走，除了一把旧提琴。</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n"/>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>ev.rev.title</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>圣西尔万堡垒</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n"/>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>ev.rev.p1</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>起义的旗帜插上了圣西尔万堡垒的残垣。</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n"/>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>ev.rev.p2</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>艾德里安倒在城墙下，手里还攥着那枚旧坠子。</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n"/>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>ev.rev.p3</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>多年以后，人们把这一天写进了教科书。</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n"/>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>ev.musician.title</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>多年以后</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n"/>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>ev.musician.p1</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>多年以后，邻国的音乐厅里，一位女提琴手正在演奏一首无人听过的曲子。</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n"/>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>ev.musician.p2</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>有人问她这首曲子叫什么。她说：「《奥尔狄亚的春天》。」</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n"/>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>ev.world.day3.title</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>第三日的晨报</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>保留原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n"/>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>ev.world.day3.p1</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>街口传来报童的声音：商队今天抵达。</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>保留原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n"/>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>ev.world.day3.p2</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>咖啡馆里多了一些陌生面孔，老陈擦亮了门前的招牌。</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>保留原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n"/>
+      <c r="B90" s="2" t="inlineStr">
         <is>
           <t>mainmenu.title</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C90" s="3" t="inlineStr">
         <is>
           <t>银星劫</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D90" s="2" t="inlineStr">
         <is>
           <t>主菜单标题</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr"/>
-      <c r="B6" s="3" t="inlineStr">
+    <row r="91">
+      <c r="A91" s="2" t="n"/>
+      <c r="B91" s="2" t="inlineStr">
         <is>
           <t>mainmenu.subtitle</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C91" s="3" t="inlineStr">
         <is>
           <t>文本由 Luban Excel 注入</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>文本配表示例说明</t>
+      <c r="D91" s="2" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n"/>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>npc.chen.name</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>老陈</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n"/>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>npc.chen.desc</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>守着咖啡馆的老陈。</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n"/>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>ev.chen.tea.title</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>老陈递来一杯茶</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n"/>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>ev.chen.tea.p1</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>“喝口茶吧。”</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n"/>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>ev.chen.tea.p2</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>屋里的灯光暖了些。</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n"/>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>bar.trust.name</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>信任</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n"/>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>bar.willpower.name</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>意志</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n"/>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>choice.tea.accept</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>接过茶杯</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>原示例</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Save current cafe progress
</commit_message>
<xml_diff>
--- a/Assets/ConfigTables/Data/Text.xlsx
+++ b/Assets/ConfigTables/Data/Text.xlsx
@@ -1,40 +1,198 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="29520" windowHeight="14100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Text" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Text" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="23">
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
       <i val="1"/>
-      <color rgb="00666666"/>
+      <color rgb="FF666666"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
       <patternFill/>
     </fill>
@@ -43,11 +201,198 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004F81BD"/>
+        <fgColor rgb="FF4F81BD"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -55,11 +400,268 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -70,9 +672,62 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="49">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -425,7 +1080,6 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -435,13 +1089,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D111"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" style="6" min="1" max="1"/>
+    <col width="28" customWidth="1" style="6" min="2" max="2"/>
+    <col width="36" customWidth="1" style="6" min="3" max="3"/>
+    <col width="28" customWidth="1" style="6" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -772,6 +1426,1444 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="4" t="n"/>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>npc.a.name</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>艾德里安</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>A · 短工佣人，出身寒微</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28.8" customHeight="1" s="6">
+      <c r="A20" s="4" t="n"/>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>npc.a.desc</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>在王都打短工的年轻人，读过几本禁书。</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>A 角色描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n"/>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>npc.b.name</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>塞西莉亚</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>B · 没落王选者家的小姐</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28.8" customHeight="1" s="6">
+      <c r="A22" s="4" t="n"/>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>npc.b.desc</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>家道中落的贵族小姐，不甘于被安排的婚事。</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>B 角色描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n"/>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>npc.c.name</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>朱利安</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>C · 普通王选者家族的少爷</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28.8" customHeight="1" s="6">
+      <c r="A24" s="4" t="n"/>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>npc.c.desc</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>出身体面的年轻贵族，一心想娶塞西莉亚。</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>C 角色描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n"/>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>npc.d.name</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>老伯爵瓦尔蒙</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>D · 塞西莉亚的父亲</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28.8" customHeight="1" s="6">
+      <c r="A26" s="4" t="n"/>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>npc.d.desc</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>固执的旧贵族，把家族的体面看得比女儿重要。</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>D 角色描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n"/>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>player.name</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>你</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>玩家 · 咖啡馆的旁观者</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="28.8" customHeight="1" s="6">
+      <c r="A28" s="4" t="n"/>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>player.desc</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>你坐在咖啡馆的角落，看着这一切发生。你可以插手，也可以只是看着。</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>玩家描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n"/>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>world.name</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>奥尔狄亚王国</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>世界观</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="28.8" customHeight="1" s="6">
+      <c r="A30" s="4" t="n"/>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>world.desc</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>一个王权将倾的王国。咖啡馆里，新旧思想正在交锋。</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>世界描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n"/>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>bar.a.thought.name</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>进步思想</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>A 的思想觉悟</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n"/>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>bar.a.trust_b.name</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>A对B的爱慕</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>A 对 B 的感情</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n"/>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>bar.a.respect_c.name</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>A对C的敬服</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>A 对 C 的态度</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n"/>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>bar.b.trust_a.name</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>B对A的爱慕</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>B 对 A 的感情</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n"/>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>bar.b.trust_c.name</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>B对C的情谊</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>B 对 C 的感情</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n"/>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>bar.b.trust_d.name</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>B对父亲的信任</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>B 对 D 的信任</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n"/>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>bar.b.rebel.name</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>B的叛逆</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>B 的叛逆程度</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n"/>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>bar.c.wealth.name</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>C的家产</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>C 的家产与地位</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n"/>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>bar.c.trust_b.name</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>C对B的爱慕</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>C 对 B 的感情</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="n"/>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>bar.stability.name</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>王国稳定</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>王国的稳定程度</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n"/>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>bar.calendar.name</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>第几天</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n"/>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>ev.act.meet.title</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>咖啡馆的私语</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43" ht="28.8" customHeight="1" s="6">
+      <c r="A43" s="4" t="n"/>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>ev.act.meet.p1</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>你替艾德里安和塞西莉亚在咖啡馆后座留了位置。</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44" ht="28.8" customHeight="1" s="6">
+      <c r="A44" s="4" t="n"/>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>ev.act.meet.p2</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>两人说了很久的话。离开时，塞西莉亚的脸上有一点笑意。</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n"/>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>ev.act.cwithb.title</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>让让他们独处</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46" ht="28.8" customHeight="1" s="6">
+      <c r="A46" s="4" t="n"/>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>ev.act.cwithb.p1</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>你替朱利安制造了一个和塞西莉亚独处的下午。</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47" ht="28.8" customHeight="1" s="6">
+      <c r="A47" s="4" t="n"/>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>ev.act.cwithb.p2</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>他讲了些得体的笑话，塞西莉亚礼貌地听着。</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="n"/>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>ev.act.salon.title</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>改革派沙龙</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n"/>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>ev.act.salon.p1</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>你把艾德里安带进了改革派的沙龙。</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50" ht="28.8" customHeight="1" s="6">
+      <c r="A50" s="4" t="n"/>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>ev.act.salon.p2</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>他听得很认真，末了问了一句让全场安静下来的话。</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="n"/>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>ev.act.peer.title</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>伯爵的关系</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="n"/>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>ev.act.peer.p1</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>你替朱利安搭上了伯爵的门路。</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="n"/>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>ev.act.peer.p2</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>一个月后，他谋到了一个体面的职位。</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="n"/>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>ev.talk.cafe.title</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>咖啡馆的午后</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr"/>
+    </row>
+    <row r="55" ht="43.2" customHeight="1" s="6">
+      <c r="A55" s="4" t="n"/>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>ev.talk.cafe.p1</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>塞西莉亚坐在窗边，用勺子搅着已经凉掉的咖啡。她说：「你说，人是不是只能过一种人生。」</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="n"/>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>choice.talk.cafe.a</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>「你可以选别人没走过的那条。」</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="n"/>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>choice.talk.cafe.b</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>「回去吧，别让你父亲担心。」</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="n"/>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>choice.talk.cafe.c</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>「时代要变了，你我都看得见。」</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="n"/>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>ev.ab.swear.title</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>私定终生</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr"/>
+    </row>
+    <row r="60" ht="28.8" customHeight="1" s="6">
+      <c r="A60" s="4" t="n"/>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>ev.ab.swear.p1</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>塞西莉亚摘下颈上那枚旧坠子，塞进艾德里安手里。</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="n"/>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>ev.ab.swear.p2</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>「等春天，我们就走。」</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr"/>
+    </row>
+    <row r="62" ht="28.8" customHeight="1" s="6">
+      <c r="A62" s="4" t="n"/>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>ev.ab.swear.p3</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>咖啡馆的灯影在窗上晃了一下，谁也没有再说话。</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="n"/>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>ev.bc.swear.title</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>门当户对</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr"/>
+    </row>
+    <row r="64" ht="28.8" customHeight="1" s="6">
+      <c r="A64" s="4" t="n"/>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>ev.bc.swear.p1</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>朱利安跪在塞西莉亚面前，捧出家族的戒指。</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="n"/>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>ev.bc.swear.p2</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>「我会给你一个体面的家。」</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="n"/>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>ev.bc.swear.p3</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>塞西莉亚看了很久，最后点了点头。</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="n"/>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>ev.standoff.title</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>三人的对峙</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr"/>
+    </row>
+    <row r="68" ht="28.8" customHeight="1" s="6">
+      <c r="A68" s="4" t="n"/>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>ev.standoff.p1</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>咖啡馆打烊了，只剩下三个人和一盏灯。</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr"/>
+    </row>
+    <row r="69" ht="28.8" customHeight="1" s="6">
+      <c r="A69" s="4" t="n"/>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>ev.standoff.p2</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>「你凭什么？」朱利安说。艾德里安没有回答。</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="n"/>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>ev.standoff.p3</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>塞西莉亚站在中间，谁也没有看。</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="n"/>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>ev.comrade.title</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>同志</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr"/>
+    </row>
+    <row r="72" ht="28.8" customHeight="1" s="6">
+      <c r="A72" s="4" t="n"/>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>ev.comrade.p1</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>艾德里安把一本小册子推到朱利安面前。</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr"/>
+    </row>
+    <row r="73" ht="28.8" customHeight="1" s="6">
+      <c r="A73" s="4" t="n"/>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>ev.comrade.p2</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>朱利安读了一夜。天亮时他说：「你说得对。」</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="n"/>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>ev.prison.title</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>冤狱</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr"/>
+    </row>
+    <row r="75" ht="28.8" customHeight="1" s="6">
+      <c r="A75" s="4" t="n"/>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>ev.prison.p1</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>塞西莉亚被指控窝藏禁书，押进了圣西尔万的黑牢。</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76" ht="28.8" customHeight="1" s="6">
+      <c r="A76" s="4" t="n"/>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>ev.prison.p2</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>老伯爵在门外站了很久，最终没有进去。</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="n"/>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>ev.rescue.title</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>捞人</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="n"/>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>ev.rescue.p1</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>你动用了积攒多年的关系。</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr"/>
+    </row>
+    <row r="79" ht="28.8" customHeight="1" s="6">
+      <c r="A79" s="4" t="n"/>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>ev.rescue.p2</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>三天后，塞西莉亚从牢里走了出来，瘦了一圈。</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="n"/>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>ev.dq1.title</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>第一次顶撞</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="n"/>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>ev.dq1.p1</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>「我不嫁。」塞西莉亚说。</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr"/>
+    </row>
+    <row r="82" ht="28.8" customHeight="1" s="6">
+      <c r="A82" s="4" t="n"/>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>ev.dq1.p2</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>老伯爵把茶杯顿在桌上，没有再说一个字。</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="n"/>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>ev.dq2.title</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>第二次顶撞</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="n"/>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>ev.dq2.p1</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>「你从来只想着你那个姓氏！」</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="n"/>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>ev.dq2.p2</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>这一次，塞西莉亚摔门而出。</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="n"/>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>ev.dqn.title</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>沉默的餐桌</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr"/>
+    </row>
+    <row r="87" ht="28.8" customHeight="1" s="6">
+      <c r="A87" s="4" t="n"/>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>ev.dqn.p1</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>父女二人隔着一张长桌吃饭，全程没有人开口。</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="n"/>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>ev.elope.title</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>私奔</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr"/>
+    </row>
+    <row r="89" ht="28.8" customHeight="1" s="6">
+      <c r="A89" s="4" t="n"/>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>ev.elope.p1</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>没有婚礼，没有嫁妆。两个人趁着夜色出了城门。</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr"/>
+    </row>
+    <row r="90" ht="28.8" customHeight="1" s="6">
+      <c r="A90" s="4" t="n"/>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>ev.elope.p2</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>塞西莉亚回头看了一眼，老伯爵的宅邸没有一盏灯是亮的。</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="n"/>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>ev.flee.title</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>家族的出走</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr"/>
+    </row>
+    <row r="92" ht="28.8" customHeight="1" s="6">
+      <c r="A92" s="4" t="n"/>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>ev.flee.p1</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>恐怖统治的前夜，瓦尔蒙一家收拾了细软，连夜离开了奥尔狄亚。</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr"/>
+    </row>
+    <row r="93" ht="28.8" customHeight="1" s="6">
+      <c r="A93" s="4" t="n"/>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>ev.flee.p2</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>塞西莉亚什么也没带走，除了一把旧提琴。</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="n"/>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>ev.rev.title</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>圣西尔万堡垒</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr"/>
+    </row>
+    <row r="95" ht="28.8" customHeight="1" s="6">
+      <c r="A95" s="4" t="n"/>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>ev.rev.p1</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>起义的旗帜插上了圣西尔万堡垒的残垣。</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr"/>
+    </row>
+    <row r="96" ht="28.8" customHeight="1" s="6">
+      <c r="A96" s="4" t="n"/>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>ev.rev.p2</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>艾德里安倒在城墙下，手里还攥着那枚旧坠子。</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr"/>
+    </row>
+    <row r="97" ht="28.8" customHeight="1" s="6">
+      <c r="A97" s="4" t="n"/>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>ev.rev.p3</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>多年以后，人们把这一天写进了教科书。</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="n"/>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>ev.musician.title</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>多年以后</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr"/>
+    </row>
+    <row r="99" ht="28.8" customHeight="1" s="6">
+      <c r="A99" s="4" t="n"/>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>ev.musician.p1</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>多年以后，邻国的音乐厅里，一位女提琴手正在演奏一首无人听过的曲子。</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr"/>
+    </row>
+    <row r="100" ht="28.8" customHeight="1" s="6">
+      <c r="A100" s="4" t="n"/>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>ev.musician.p2</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>有人问她这首曲子叫什么。她说：「《奥尔狄亚的春天》。」</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="n"/>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>ev.world.day3.title</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>第三日的晨报</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr">
+        <is>
+          <t>保留原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="n"/>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>ev.world.day3.p1</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>街口传来报童的声音：商队今天抵达。</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>保留原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="28.8" customHeight="1" s="6">
+      <c r="A103" s="4" t="n"/>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>ev.world.day3.p2</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>咖啡馆里多了一些陌生面孔，老陈擦亮了门前的招牌。</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr">
+        <is>
+          <t>保留原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="n"/>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>npc.chen.name</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>老陈</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="n"/>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>npc.chen.desc</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>守着咖啡馆的老陈。</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="n"/>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>ev.chen.tea.title</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>老陈递来一杯茶</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="n"/>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>ev.chen.tea.p1</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>“喝口茶吧。”</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
+          <t>原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="n"/>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>ev.chen.tea.p2</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>屋里的灯光暖了些。</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="n"/>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>bar.trust.name</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>信任</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="4" t="n"/>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>bar.willpower.name</t>
+        </is>
+      </c>
+      <c r="C110" s="5" t="inlineStr">
+        <is>
+          <t>意志</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>原示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="n"/>
+      <c r="B111" s="4" t="inlineStr">
+        <is>
+          <t>choice.tea.accept</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>接过茶杯</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>原示例</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>